<commit_message>
update price 12-18 mar
</commit_message>
<xml_diff>
--- a/database/1/7. 3339 - ANYDAY LADIES.XLSX
+++ b/database/1/7. 3339 - ANYDAY LADIES.XLSX
@@ -2100,10 +2100,10 @@
         <v>275</v>
       </c>
       <c r="B2" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C2" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D2" s="5">
         <v>3339</v>
@@ -2151,10 +2151,10 @@
         <v>275</v>
       </c>
       <c r="B3" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C3" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D3" s="5">
         <v>3339</v>
@@ -2202,10 +2202,10 @@
         <v>275</v>
       </c>
       <c r="B4" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C4" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D4" s="5">
         <v>3339</v>
@@ -2253,10 +2253,10 @@
         <v>275</v>
       </c>
       <c r="B5" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C5" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D5" s="5">
         <v>3339</v>
@@ -2304,10 +2304,10 @@
         <v>275</v>
       </c>
       <c r="B6" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C6" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D6" s="5">
         <v>3339</v>
@@ -2355,10 +2355,10 @@
         <v>275</v>
       </c>
       <c r="B7" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C7" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D7" s="5">
         <v>3339</v>
@@ -2406,10 +2406,10 @@
         <v>275</v>
       </c>
       <c r="B8" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C8" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D8" s="5">
         <v>3339</v>
@@ -2457,10 +2457,10 @@
         <v>275</v>
       </c>
       <c r="B9" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C9" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D9" s="5">
         <v>3339</v>
@@ -2508,10 +2508,10 @@
         <v>275</v>
       </c>
       <c r="B10" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C10" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D10" s="5">
         <v>3339</v>
@@ -2559,10 +2559,10 @@
         <v>275</v>
       </c>
       <c r="B11" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C11" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D11" s="5">
         <v>3339</v>
@@ -2610,10 +2610,10 @@
         <v>275</v>
       </c>
       <c r="B12" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C12" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D12" s="5">
         <v>3339</v>
@@ -2661,10 +2661,10 @@
         <v>275</v>
       </c>
       <c r="B13" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C13" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D13" s="5">
         <v>3339</v>
@@ -2712,10 +2712,10 @@
         <v>275</v>
       </c>
       <c r="B14" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C14" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D14" s="5">
         <v>3339</v>
@@ -2763,10 +2763,10 @@
         <v>275</v>
       </c>
       <c r="B15" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C15" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D15" s="5">
         <v>3339</v>
@@ -2814,10 +2814,10 @@
         <v>275</v>
       </c>
       <c r="B16" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C16" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D16" s="5">
         <v>3339</v>
@@ -2865,10 +2865,10 @@
         <v>275</v>
       </c>
       <c r="B17" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C17" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D17" s="5">
         <v>3339</v>
@@ -2916,10 +2916,10 @@
         <v>275</v>
       </c>
       <c r="B18" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C18" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D18" s="5">
         <v>3339</v>
@@ -2967,10 +2967,10 @@
         <v>275</v>
       </c>
       <c r="B19" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C19" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D19" s="5">
         <v>3339</v>
@@ -3018,10 +3018,10 @@
         <v>275</v>
       </c>
       <c r="B20" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C20" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D20" s="5">
         <v>3339</v>
@@ -3069,10 +3069,10 @@
         <v>275</v>
       </c>
       <c r="B21" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C21" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D21" s="5">
         <v>3339</v>
@@ -3120,10 +3120,10 @@
         <v>275</v>
       </c>
       <c r="B22" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C22" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D22" s="5">
         <v>3339</v>
@@ -3171,10 +3171,10 @@
         <v>275</v>
       </c>
       <c r="B23" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C23" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D23" s="5">
         <v>3339</v>
@@ -3222,10 +3222,10 @@
         <v>275</v>
       </c>
       <c r="B24" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C24" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D24" s="5">
         <v>3339</v>
@@ -3273,10 +3273,10 @@
         <v>275</v>
       </c>
       <c r="B25" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C25" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D25" s="5">
         <v>3339</v>
@@ -3324,10 +3324,10 @@
         <v>275</v>
       </c>
       <c r="B26" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C26" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D26" s="5">
         <v>3339</v>
@@ -3375,10 +3375,10 @@
         <v>275</v>
       </c>
       <c r="B27" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C27" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D27" s="5">
         <v>3339</v>
@@ -3426,10 +3426,10 @@
         <v>275</v>
       </c>
       <c r="B28" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C28" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D28" s="5">
         <v>3339</v>
@@ -3477,10 +3477,10 @@
         <v>275</v>
       </c>
       <c r="B29" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C29" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D29" s="5">
         <v>3339</v>
@@ -3528,10 +3528,10 @@
         <v>275</v>
       </c>
       <c r="B30" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C30" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D30" s="5">
         <v>3339</v>
@@ -3579,10 +3579,10 @@
         <v>275</v>
       </c>
       <c r="B31" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C31" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D31" s="5">
         <v>3339</v>
@@ -3630,10 +3630,10 @@
         <v>275</v>
       </c>
       <c r="B32" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C32" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D32" s="5">
         <v>3339</v>
@@ -3681,10 +3681,10 @@
         <v>275</v>
       </c>
       <c r="B33" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C33" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D33" s="5">
         <v>3339</v>
@@ -3732,10 +3732,10 @@
         <v>275</v>
       </c>
       <c r="B34" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C34" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D34" s="5">
         <v>3339</v>
@@ -3783,10 +3783,10 @@
         <v>275</v>
       </c>
       <c r="B35" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C35" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D35" s="5">
         <v>3339</v>
@@ -3834,10 +3834,10 @@
         <v>275</v>
       </c>
       <c r="B36" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C36" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D36" s="5">
         <v>3339</v>
@@ -3885,10 +3885,10 @@
         <v>275</v>
       </c>
       <c r="B37" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C37" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D37" s="5">
         <v>3339</v>
@@ -3936,10 +3936,10 @@
         <v>275</v>
       </c>
       <c r="B38" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C38" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D38" s="5">
         <v>3339</v>
@@ -3987,10 +3987,10 @@
         <v>275</v>
       </c>
       <c r="B39" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C39" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D39" s="5">
         <v>3339</v>
@@ -4038,10 +4038,10 @@
         <v>275</v>
       </c>
       <c r="B40" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C40" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D40" s="5">
         <v>3339</v>
@@ -4089,10 +4089,10 @@
         <v>275</v>
       </c>
       <c r="B41" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C41" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D41" s="5">
         <v>3339</v>
@@ -4140,10 +4140,10 @@
         <v>275</v>
       </c>
       <c r="B42" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C42" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D42" s="5">
         <v>3339</v>
@@ -4191,10 +4191,10 @@
         <v>275</v>
       </c>
       <c r="B43" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C43" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D43" s="5">
         <v>3339</v>
@@ -4242,10 +4242,10 @@
         <v>275</v>
       </c>
       <c r="B44" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C44" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D44" s="5">
         <v>3339</v>
@@ -4293,10 +4293,10 @@
         <v>275</v>
       </c>
       <c r="B45" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C45" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D45" s="5">
         <v>3339</v>
@@ -4344,10 +4344,10 @@
         <v>275</v>
       </c>
       <c r="B46" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C46" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D46" s="5">
         <v>3339</v>
@@ -4395,10 +4395,10 @@
         <v>275</v>
       </c>
       <c r="B47" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C47" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D47" s="5">
         <v>3339</v>
@@ -4446,10 +4446,10 @@
         <v>275</v>
       </c>
       <c r="B48" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C48" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D48" s="5">
         <v>3339</v>
@@ -4497,10 +4497,10 @@
         <v>275</v>
       </c>
       <c r="B49" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C49" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D49" s="5">
         <v>3339</v>
@@ -4548,10 +4548,10 @@
         <v>275</v>
       </c>
       <c r="B50" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C50" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D50" s="5">
         <v>3339</v>
@@ -4599,10 +4599,10 @@
         <v>275</v>
       </c>
       <c r="B51" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C51" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D51" s="5">
         <v>3339</v>
@@ -4650,10 +4650,10 @@
         <v>275</v>
       </c>
       <c r="B52" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C52" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D52" s="5">
         <v>3339</v>
@@ -4701,10 +4701,10 @@
         <v>275</v>
       </c>
       <c r="B53" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C53" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D53" s="5">
         <v>3339</v>
@@ -4752,10 +4752,10 @@
         <v>275</v>
       </c>
       <c r="B54" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C54" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D54" s="5">
         <v>3339</v>
@@ -4803,10 +4803,10 @@
         <v>275</v>
       </c>
       <c r="B55" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C55" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D55" s="5">
         <v>3339</v>
@@ -4854,10 +4854,10 @@
         <v>275</v>
       </c>
       <c r="B56" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C56" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D56" s="5">
         <v>3339</v>
@@ -4905,10 +4905,10 @@
         <v>275</v>
       </c>
       <c r="B57" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C57" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D57" s="5">
         <v>3339</v>
@@ -4956,10 +4956,10 @@
         <v>275</v>
       </c>
       <c r="B58" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C58" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D58" s="5">
         <v>3339</v>
@@ -5007,10 +5007,10 @@
         <v>275</v>
       </c>
       <c r="B59" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C59" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D59" s="5">
         <v>3339</v>
@@ -5058,10 +5058,10 @@
         <v>275</v>
       </c>
       <c r="B60" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C60" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D60" s="5">
         <v>3339</v>
@@ -5109,10 +5109,10 @@
         <v>275</v>
       </c>
       <c r="B61" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C61" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D61" s="5">
         <v>3339</v>
@@ -5160,10 +5160,10 @@
         <v>275</v>
       </c>
       <c r="B62" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C62" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D62" s="5">
         <v>3339</v>
@@ -5211,10 +5211,10 @@
         <v>275</v>
       </c>
       <c r="B63" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C63" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D63" s="5">
         <v>3339</v>
@@ -5262,10 +5262,10 @@
         <v>275</v>
       </c>
       <c r="B64" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C64" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D64" s="5">
         <v>3339</v>
@@ -5313,10 +5313,10 @@
         <v>275</v>
       </c>
       <c r="B65" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C65" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D65" s="5">
         <v>3339</v>
@@ -5364,10 +5364,10 @@
         <v>275</v>
       </c>
       <c r="B66" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C66" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D66" s="5">
         <v>3339</v>
@@ -5415,10 +5415,10 @@
         <v>275</v>
       </c>
       <c r="B67" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C67" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D67" s="5">
         <v>3339</v>
@@ -5466,10 +5466,10 @@
         <v>275</v>
       </c>
       <c r="B68" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C68" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D68" s="5">
         <v>3339</v>
@@ -5517,10 +5517,10 @@
         <v>275</v>
       </c>
       <c r="B69" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C69" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D69" s="5">
         <v>3339</v>
@@ -5568,10 +5568,10 @@
         <v>275</v>
       </c>
       <c r="B70" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C70" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D70" s="5">
         <v>3339</v>
@@ -5619,10 +5619,10 @@
         <v>275</v>
       </c>
       <c r="B71" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C71" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D71" s="5">
         <v>3339</v>
@@ -5670,10 +5670,10 @@
         <v>275</v>
       </c>
       <c r="B72" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C72" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D72" s="5">
         <v>3339</v>
@@ -5721,10 +5721,10 @@
         <v>275</v>
       </c>
       <c r="B73" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C73" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D73" s="5">
         <v>3339</v>
@@ -5772,10 +5772,10 @@
         <v>275</v>
       </c>
       <c r="B74" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C74" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D74" s="5">
         <v>3339</v>
@@ -5823,10 +5823,10 @@
         <v>275</v>
       </c>
       <c r="B75" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C75" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D75" s="5">
         <v>3339</v>
@@ -5874,10 +5874,10 @@
         <v>275</v>
       </c>
       <c r="B76" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C76" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D76" s="5">
         <v>3339</v>
@@ -5925,10 +5925,10 @@
         <v>275</v>
       </c>
       <c r="B77" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C77" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D77" s="5">
         <v>3339</v>
@@ -5976,10 +5976,10 @@
         <v>275</v>
       </c>
       <c r="B78" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C78" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D78" s="5">
         <v>3339</v>
@@ -6027,10 +6027,10 @@
         <v>275</v>
       </c>
       <c r="B79" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C79" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D79" s="5">
         <v>3339</v>
@@ -6078,10 +6078,10 @@
         <v>275</v>
       </c>
       <c r="B80" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C80" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D80" s="5">
         <v>3339</v>
@@ -6129,10 +6129,10 @@
         <v>275</v>
       </c>
       <c r="B81" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C81" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D81" s="5">
         <v>3339</v>
@@ -6180,10 +6180,10 @@
         <v>275</v>
       </c>
       <c r="B82" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C82" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D82" s="5">
         <v>3339</v>
@@ -6231,10 +6231,10 @@
         <v>275</v>
       </c>
       <c r="B83" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C83" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D83" s="5">
         <v>3339</v>
@@ -6282,10 +6282,10 @@
         <v>275</v>
       </c>
       <c r="B84" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C84" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D84" s="5">
         <v>3339</v>
@@ -6333,10 +6333,10 @@
         <v>275</v>
       </c>
       <c r="B85" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C85" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D85" s="5">
         <v>3339</v>
@@ -6384,10 +6384,10 @@
         <v>275</v>
       </c>
       <c r="B86" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C86" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D86" s="5">
         <v>3339</v>
@@ -6435,10 +6435,10 @@
         <v>275</v>
       </c>
       <c r="B87" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C87" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D87" s="5">
         <v>3339</v>
@@ -6486,10 +6486,10 @@
         <v>275</v>
       </c>
       <c r="B88" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C88" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D88" s="5">
         <v>3339</v>
@@ -6537,10 +6537,10 @@
         <v>275</v>
       </c>
       <c r="B89" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C89" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D89" s="5">
         <v>3339</v>
@@ -6588,10 +6588,10 @@
         <v>275</v>
       </c>
       <c r="B90" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C90" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D90" s="5">
         <v>3339</v>
@@ -6639,10 +6639,10 @@
         <v>275</v>
       </c>
       <c r="B91" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C91" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D91" s="5">
         <v>3339</v>
@@ -6690,10 +6690,10 @@
         <v>275</v>
       </c>
       <c r="B92" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C92" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D92" s="5">
         <v>3339</v>
@@ -6741,10 +6741,10 @@
         <v>275</v>
       </c>
       <c r="B93" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C93" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D93" s="5">
         <v>3339</v>
@@ -6792,10 +6792,10 @@
         <v>275</v>
       </c>
       <c r="B94" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C94" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D94" s="5">
         <v>3339</v>
@@ -6843,10 +6843,10 @@
         <v>275</v>
       </c>
       <c r="B95" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C95" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D95" s="5">
         <v>3339</v>
@@ -6894,10 +6894,10 @@
         <v>275</v>
       </c>
       <c r="B96" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C96" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D96" s="5">
         <v>3339</v>
@@ -6945,10 +6945,10 @@
         <v>275</v>
       </c>
       <c r="B97" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C97" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D97" s="5">
         <v>3339</v>
@@ -6996,10 +6996,10 @@
         <v>275</v>
       </c>
       <c r="B98" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C98" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D98" s="5">
         <v>3339</v>
@@ -7047,10 +7047,10 @@
         <v>275</v>
       </c>
       <c r="B99" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C99" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D99" s="5">
         <v>3339</v>
@@ -7098,10 +7098,10 @@
         <v>275</v>
       </c>
       <c r="B100" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C100" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D100" s="5">
         <v>3339</v>
@@ -7149,10 +7149,10 @@
         <v>275</v>
       </c>
       <c r="B101" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C101" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D101" s="5">
         <v>3339</v>
@@ -7282,10 +7282,10 @@
         <v>274</v>
       </c>
       <c r="B2" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C2" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D2" s="5">
         <v>3339</v>
@@ -7333,10 +7333,10 @@
         <v>274</v>
       </c>
       <c r="B3" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C3" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D3" s="5">
         <v>3339</v>
@@ -7384,10 +7384,10 @@
         <v>274</v>
       </c>
       <c r="B4" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C4" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D4" s="5">
         <v>3339</v>
@@ -7435,10 +7435,10 @@
         <v>274</v>
       </c>
       <c r="B5" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C5" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D5" s="5">
         <v>3339</v>
@@ -7486,10 +7486,10 @@
         <v>274</v>
       </c>
       <c r="B6" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C6" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D6" s="5">
         <v>3339</v>
@@ -7537,10 +7537,10 @@
         <v>274</v>
       </c>
       <c r="B7" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C7" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D7" s="5">
         <v>3339</v>
@@ -7588,10 +7588,10 @@
         <v>274</v>
       </c>
       <c r="B8" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C8" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D8" s="5">
         <v>3339</v>
@@ -7639,10 +7639,10 @@
         <v>274</v>
       </c>
       <c r="B9" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C9" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D9" s="5">
         <v>3339</v>
@@ -7690,10 +7690,10 @@
         <v>274</v>
       </c>
       <c r="B10" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C10" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D10" s="5">
         <v>3339</v>
@@ -7741,10 +7741,10 @@
         <v>274</v>
       </c>
       <c r="B11" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C11" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D11" s="5">
         <v>3339</v>
@@ -7792,10 +7792,10 @@
         <v>274</v>
       </c>
       <c r="B12" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C12" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D12" s="5">
         <v>3339</v>
@@ -7843,10 +7843,10 @@
         <v>274</v>
       </c>
       <c r="B13" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C13" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D13" s="5">
         <v>3339</v>
@@ -7894,10 +7894,10 @@
         <v>274</v>
       </c>
       <c r="B14" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C14" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D14" s="5">
         <v>3339</v>
@@ -7945,10 +7945,10 @@
         <v>274</v>
       </c>
       <c r="B15" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C15" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D15" s="5">
         <v>3339</v>
@@ -7996,10 +7996,10 @@
         <v>274</v>
       </c>
       <c r="B16" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C16" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D16" s="5">
         <v>3339</v>
@@ -8047,10 +8047,10 @@
         <v>274</v>
       </c>
       <c r="B17" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C17" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D17" s="5">
         <v>3339</v>
@@ -8098,10 +8098,10 @@
         <v>274</v>
       </c>
       <c r="B18" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C18" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D18" s="5">
         <v>3339</v>
@@ -8149,10 +8149,10 @@
         <v>274</v>
       </c>
       <c r="B19" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C19" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D19" s="5">
         <v>3339</v>
@@ -8200,10 +8200,10 @@
         <v>274</v>
       </c>
       <c r="B20" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C20" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D20" s="5">
         <v>3339</v>
@@ -8251,10 +8251,10 @@
         <v>274</v>
       </c>
       <c r="B21" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C21" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D21" s="5">
         <v>3339</v>
@@ -8302,10 +8302,10 @@
         <v>274</v>
       </c>
       <c r="B22" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C22" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D22" s="5">
         <v>3339</v>
@@ -8353,10 +8353,10 @@
         <v>274</v>
       </c>
       <c r="B23" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C23" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D23" s="5">
         <v>3339</v>
@@ -8404,10 +8404,10 @@
         <v>274</v>
       </c>
       <c r="B24" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C24" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D24" s="5">
         <v>3339</v>
@@ -8455,10 +8455,10 @@
         <v>274</v>
       </c>
       <c r="B25" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C25" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D25" s="5">
         <v>3339</v>
@@ -8506,10 +8506,10 @@
         <v>274</v>
       </c>
       <c r="B26" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C26" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D26" s="5">
         <v>3339</v>
@@ -8557,10 +8557,10 @@
         <v>274</v>
       </c>
       <c r="B27" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C27" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D27" s="5">
         <v>3339</v>
@@ -8608,10 +8608,10 @@
         <v>274</v>
       </c>
       <c r="B28" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C28" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D28" s="5">
         <v>3339</v>
@@ -8659,10 +8659,10 @@
         <v>274</v>
       </c>
       <c r="B29" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C29" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D29" s="5">
         <v>3339</v>
@@ -8710,10 +8710,10 @@
         <v>274</v>
       </c>
       <c r="B30" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C30" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D30" s="5">
         <v>3339</v>
@@ -8761,10 +8761,10 @@
         <v>274</v>
       </c>
       <c r="B31" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C31" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D31" s="5">
         <v>3339</v>
@@ -8812,10 +8812,10 @@
         <v>274</v>
       </c>
       <c r="B32" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C32" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D32" s="5">
         <v>3339</v>
@@ -8863,10 +8863,10 @@
         <v>274</v>
       </c>
       <c r="B33" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C33" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D33" s="5">
         <v>3339</v>
@@ -8914,10 +8914,10 @@
         <v>274</v>
       </c>
       <c r="B34" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C34" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D34" s="5">
         <v>3339</v>
@@ -8965,10 +8965,10 @@
         <v>274</v>
       </c>
       <c r="B35" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C35" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D35" s="5">
         <v>3339</v>
@@ -9016,10 +9016,10 @@
         <v>274</v>
       </c>
       <c r="B36" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C36" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D36" s="5">
         <v>3339</v>
@@ -9067,10 +9067,10 @@
         <v>274</v>
       </c>
       <c r="B37" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C37" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D37" s="5">
         <v>3339</v>
@@ -9118,10 +9118,10 @@
         <v>274</v>
       </c>
       <c r="B38" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C38" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D38" s="5">
         <v>3339</v>
@@ -9169,10 +9169,10 @@
         <v>274</v>
       </c>
       <c r="B39" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C39" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D39" s="5">
         <v>3339</v>
@@ -9220,10 +9220,10 @@
         <v>274</v>
       </c>
       <c r="B40" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C40" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D40" s="5">
         <v>3339</v>
@@ -9271,10 +9271,10 @@
         <v>274</v>
       </c>
       <c r="B41" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C41" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D41" s="5">
         <v>3339</v>
@@ -9322,10 +9322,10 @@
         <v>274</v>
       </c>
       <c r="B42" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C42" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D42" s="5">
         <v>3339</v>
@@ -9373,10 +9373,10 @@
         <v>274</v>
       </c>
       <c r="B43" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C43" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D43" s="5">
         <v>3339</v>
@@ -9424,10 +9424,10 @@
         <v>274</v>
       </c>
       <c r="B44" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C44" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D44" s="5">
         <v>3339</v>
@@ -9475,10 +9475,10 @@
         <v>274</v>
       </c>
       <c r="B45" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C45" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D45" s="5">
         <v>3339</v>
@@ -9526,10 +9526,10 @@
         <v>274</v>
       </c>
       <c r="B46" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C46" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D46" s="5">
         <v>3339</v>
@@ -9577,10 +9577,10 @@
         <v>274</v>
       </c>
       <c r="B47" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C47" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D47" s="5">
         <v>3339</v>
@@ -9628,10 +9628,10 @@
         <v>274</v>
       </c>
       <c r="B48" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C48" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D48" s="5">
         <v>3339</v>
@@ -9679,10 +9679,10 @@
         <v>274</v>
       </c>
       <c r="B49" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C49" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D49" s="5">
         <v>3339</v>
@@ -9730,10 +9730,10 @@
         <v>274</v>
       </c>
       <c r="B50" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C50" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D50" s="5">
         <v>3339</v>
@@ -9781,10 +9781,10 @@
         <v>274</v>
       </c>
       <c r="B51" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C51" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D51" s="5">
         <v>3339</v>
@@ -9832,10 +9832,10 @@
         <v>274</v>
       </c>
       <c r="B52" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C52" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D52" s="5">
         <v>3339</v>
@@ -9883,10 +9883,10 @@
         <v>274</v>
       </c>
       <c r="B53" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C53" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D53" s="5">
         <v>3339</v>
@@ -9934,10 +9934,10 @@
         <v>274</v>
       </c>
       <c r="B54" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C54" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D54" s="5">
         <v>3339</v>
@@ -9985,10 +9985,10 @@
         <v>274</v>
       </c>
       <c r="B55" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C55" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D55" s="5">
         <v>3339</v>
@@ -10036,10 +10036,10 @@
         <v>274</v>
       </c>
       <c r="B56" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C56" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D56" s="5">
         <v>3339</v>
@@ -10087,10 +10087,10 @@
         <v>274</v>
       </c>
       <c r="B57" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C57" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D57" s="5">
         <v>3339</v>
@@ -10138,10 +10138,10 @@
         <v>274</v>
       </c>
       <c r="B58" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C58" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D58" s="5">
         <v>3339</v>
@@ -10189,10 +10189,10 @@
         <v>274</v>
       </c>
       <c r="B59" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C59" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D59" s="5">
         <v>3339</v>
@@ -10240,10 +10240,10 @@
         <v>274</v>
       </c>
       <c r="B60" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C60" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D60" s="5">
         <v>3339</v>
@@ -10291,10 +10291,10 @@
         <v>274</v>
       </c>
       <c r="B61" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C61" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D61" s="5">
         <v>3339</v>
@@ -10342,10 +10342,10 @@
         <v>274</v>
       </c>
       <c r="B62" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C62" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D62" s="5">
         <v>3339</v>
@@ -10393,10 +10393,10 @@
         <v>274</v>
       </c>
       <c r="B63" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C63" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D63" s="5">
         <v>3339</v>
@@ -10444,10 +10444,10 @@
         <v>274</v>
       </c>
       <c r="B64" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C64" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D64" s="5">
         <v>3339</v>
@@ -10495,10 +10495,10 @@
         <v>274</v>
       </c>
       <c r="B65" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C65" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D65" s="5">
         <v>3339</v>
@@ -10546,10 +10546,10 @@
         <v>274</v>
       </c>
       <c r="B66" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C66" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D66" s="5">
         <v>3339</v>
@@ -10597,10 +10597,10 @@
         <v>274</v>
       </c>
       <c r="B67" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C67" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D67" s="5">
         <v>3339</v>
@@ -10648,10 +10648,10 @@
         <v>274</v>
       </c>
       <c r="B68" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C68" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D68" s="5">
         <v>3339</v>
@@ -10699,10 +10699,10 @@
         <v>274</v>
       </c>
       <c r="B69" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C69" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D69" s="5">
         <v>3339</v>
@@ -10750,10 +10750,10 @@
         <v>274</v>
       </c>
       <c r="B70" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C70" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D70" s="5">
         <v>3339</v>
@@ -10801,10 +10801,10 @@
         <v>274</v>
       </c>
       <c r="B71" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C71" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D71" s="5">
         <v>3339</v>
@@ -10852,10 +10852,10 @@
         <v>274</v>
       </c>
       <c r="B72" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C72" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D72" s="5">
         <v>3339</v>
@@ -10903,10 +10903,10 @@
         <v>274</v>
       </c>
       <c r="B73" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C73" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D73" s="5">
         <v>3339</v>
@@ -10954,10 +10954,10 @@
         <v>274</v>
       </c>
       <c r="B74" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C74" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D74" s="5">
         <v>3339</v>
@@ -11005,10 +11005,10 @@
         <v>274</v>
       </c>
       <c r="B75" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C75" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D75" s="5">
         <v>3339</v>
@@ -11056,10 +11056,10 @@
         <v>274</v>
       </c>
       <c r="B76" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C76" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D76" s="5">
         <v>3339</v>
@@ -11107,10 +11107,10 @@
         <v>274</v>
       </c>
       <c r="B77" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C77" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D77" s="5">
         <v>3339</v>
@@ -11158,10 +11158,10 @@
         <v>274</v>
       </c>
       <c r="B78" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C78" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D78" s="5">
         <v>3339</v>
@@ -11209,10 +11209,10 @@
         <v>274</v>
       </c>
       <c r="B79" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C79" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D79" s="5">
         <v>3339</v>
@@ -11260,10 +11260,10 @@
         <v>274</v>
       </c>
       <c r="B80" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C80" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D80" s="5">
         <v>3339</v>
@@ -11311,10 +11311,10 @@
         <v>274</v>
       </c>
       <c r="B81" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C81" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D81" s="5">
         <v>3339</v>
@@ -11362,10 +11362,10 @@
         <v>274</v>
       </c>
       <c r="B82" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C82" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D82" s="5">
         <v>3339</v>
@@ -11413,10 +11413,10 @@
         <v>274</v>
       </c>
       <c r="B83" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C83" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D83" s="5">
         <v>3339</v>
@@ -11464,10 +11464,10 @@
         <v>274</v>
       </c>
       <c r="B84" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C84" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D84" s="5">
         <v>3339</v>
@@ -11515,10 +11515,10 @@
         <v>274</v>
       </c>
       <c r="B85" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C85" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D85" s="5">
         <v>3339</v>
@@ -11566,10 +11566,10 @@
         <v>274</v>
       </c>
       <c r="B86" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C86" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D86" s="5">
         <v>3339</v>
@@ -11617,10 +11617,10 @@
         <v>274</v>
       </c>
       <c r="B87" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C87" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D87" s="5">
         <v>3339</v>
@@ -11668,10 +11668,10 @@
         <v>274</v>
       </c>
       <c r="B88" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C88" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D88" s="5">
         <v>3339</v>
@@ -11719,10 +11719,10 @@
         <v>274</v>
       </c>
       <c r="B89" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C89" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D89" s="5">
         <v>3339</v>
@@ -11770,10 +11770,10 @@
         <v>274</v>
       </c>
       <c r="B90" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C90" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D90" s="5">
         <v>3339</v>
@@ -11821,10 +11821,10 @@
         <v>274</v>
       </c>
       <c r="B91" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C91" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D91" s="5">
         <v>3339</v>
@@ -11872,10 +11872,10 @@
         <v>274</v>
       </c>
       <c r="B92" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C92" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D92" s="5">
         <v>3339</v>
@@ -11923,10 +11923,10 @@
         <v>274</v>
       </c>
       <c r="B93" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C93" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D93" s="5">
         <v>3339</v>
@@ -11974,10 +11974,10 @@
         <v>274</v>
       </c>
       <c r="B94" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C94" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D94" s="5">
         <v>3339</v>
@@ -12025,10 +12025,10 @@
         <v>274</v>
       </c>
       <c r="B95" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C95" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D95" s="5">
         <v>3339</v>
@@ -12076,10 +12076,10 @@
         <v>274</v>
       </c>
       <c r="B96" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C96" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D96" s="5">
         <v>3339</v>
@@ -12127,10 +12127,10 @@
         <v>274</v>
       </c>
       <c r="B97" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C97" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D97" s="5">
         <v>3339</v>
@@ -12178,10 +12178,10 @@
         <v>274</v>
       </c>
       <c r="B98" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C98" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D98" s="5">
         <v>3339</v>
@@ -12229,10 +12229,10 @@
         <v>274</v>
       </c>
       <c r="B99" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C99" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D99" s="5">
         <v>3339</v>
@@ -12280,10 +12280,10 @@
         <v>274</v>
       </c>
       <c r="B100" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C100" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D100" s="5">
         <v>3339</v>
@@ -12331,10 +12331,10 @@
         <v>274</v>
       </c>
       <c r="B101" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C101" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D101" s="5">
         <v>3339</v>
@@ -12382,10 +12382,10 @@
         <v>274</v>
       </c>
       <c r="B102" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C102" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D102" s="5">
         <v>3339</v>
@@ -12433,10 +12433,10 @@
         <v>274</v>
       </c>
       <c r="B103" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C103" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D103" s="5">
         <v>3339</v>
@@ -12484,10 +12484,10 @@
         <v>274</v>
       </c>
       <c r="B104" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C104" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D104" s="5">
         <v>3339</v>
@@ -12535,10 +12535,10 @@
         <v>274</v>
       </c>
       <c r="B105" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C105" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D105" s="5">
         <v>3339</v>
@@ -12586,10 +12586,10 @@
         <v>274</v>
       </c>
       <c r="B106" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C106" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D106" s="5">
         <v>3339</v>
@@ -12637,10 +12637,10 @@
         <v>274</v>
       </c>
       <c r="B107" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C107" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D107" s="5">
         <v>3339</v>
@@ -12688,10 +12688,10 @@
         <v>274</v>
       </c>
       <c r="B108" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C108" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D108" s="5">
         <v>3339</v>
@@ -12739,10 +12739,10 @@
         <v>274</v>
       </c>
       <c r="B109" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C109" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D109" s="5">
         <v>3339</v>
@@ -12790,10 +12790,10 @@
         <v>274</v>
       </c>
       <c r="B110" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C110" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D110" s="5">
         <v>3339</v>
@@ -12841,10 +12841,10 @@
         <v>274</v>
       </c>
       <c r="B111" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C111" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D111" s="5">
         <v>3339</v>
@@ -12892,10 +12892,10 @@
         <v>274</v>
       </c>
       <c r="B112" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C112" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D112" s="5">
         <v>3339</v>
@@ -12943,10 +12943,10 @@
         <v>274</v>
       </c>
       <c r="B113" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C113" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D113" s="5">
         <v>3339</v>
@@ -12994,10 +12994,10 @@
         <v>274</v>
       </c>
       <c r="B114" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C114" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D114" s="5">
         <v>3339</v>
@@ -13045,10 +13045,10 @@
         <v>274</v>
       </c>
       <c r="B115" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C115" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D115" s="5">
         <v>3339</v>
@@ -13096,10 +13096,10 @@
         <v>274</v>
       </c>
       <c r="B116" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C116" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D116" s="5">
         <v>3339</v>
@@ -13147,10 +13147,10 @@
         <v>274</v>
       </c>
       <c r="B117" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C117" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D117" s="5">
         <v>3339</v>
@@ -13198,10 +13198,10 @@
         <v>274</v>
       </c>
       <c r="B118" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C118" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D118" s="5">
         <v>3339</v>
@@ -13249,10 +13249,10 @@
         <v>274</v>
       </c>
       <c r="B119" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C119" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D119" s="5">
         <v>3339</v>
@@ -13300,10 +13300,10 @@
         <v>274</v>
       </c>
       <c r="B120" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C120" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D120" s="5">
         <v>3339</v>
@@ -13351,10 +13351,10 @@
         <v>274</v>
       </c>
       <c r="B121" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C121" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D121" s="5">
         <v>3339</v>
@@ -13402,10 +13402,10 @@
         <v>274</v>
       </c>
       <c r="B122" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C122" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D122" s="5">
         <v>3339</v>
@@ -13453,10 +13453,10 @@
         <v>274</v>
       </c>
       <c r="B123" s="6">
-        <v>46086</v>
+        <v>46093</v>
       </c>
       <c r="C123" s="6">
-        <v>46092</v>
+        <v>46098</v>
       </c>
       <c r="D123" s="5">
         <v>3339</v>

</xml_diff>